<commit_message>
feat: novo painel escuro com glassmorphism e mapa em modo radar
</commit_message>
<xml_diff>
--- a/ROTA.xlsx
+++ b/ROTA.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>pedido</t>
   </si>
@@ -318,9 +318,7 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>0</v>
-      </c>
+      <c r="F1" s="1"/>
       <c r="G1" s="1"/>
     </row>
     <row r="2" ht="14.25" customHeight="1">

</xml_diff>